<commit_message>
Fix font errors in FRM-705 form
</commit_message>
<xml_diff>
--- a/04-Bieu-Mau/01-FRM-100/FRM-106_Pilot_Dry_Run_Log.xlsx
+++ b/04-Bieu-Mau/01-FRM-100/FRM-106_Pilot_Dry_Run_Log.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FRM106_PilotLog" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FRM106_FollowUp" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FRM106_FollowUp" sheetId="2" state="veryHidden" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FRM106_Evidence" sheetId="3" state="veryHidden" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="zLISTS" sheetId="4" state="veryHidden" r:id="rId4"/>
   </sheets>
@@ -7632,8 +7632,8 @@
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="0" insertColumns="0" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="1"/>
   <mergeCells count="95">
     <mergeCell ref="A17:G17"/>
+    <mergeCell ref="AO17:AS17"/>
     <mergeCell ref="AT13:AX13"/>
-    <mergeCell ref="AO17:AS17"/>
     <mergeCell ref="H20:O20"/>
     <mergeCell ref="AW2:BD2"/>
     <mergeCell ref="A19:G19"/>

</xml_diff>